<commit_message>
Deploy proper port binding on main app entrypoint
</commit_message>
<xml_diff>
--- a/static/attendance_sheet.xlsx
+++ b/static/attendance_sheet.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sk_sir" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="hr_sir" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="spm_sir" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="bs_sir" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="sd_sir" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sk_sir" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hr_sir" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="spm_sir" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bs_sir" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sd_sir" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teacher" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2788,4 +2789,120 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Roll No</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>101</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Abhishek</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>102</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Arpan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ashutosh</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jatin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>105</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jyotiranjan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>106</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mohit</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>107</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pranjal</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>108</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pranjul</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>109</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tarun</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update attendance template and sync project dependencies
</commit_message>
<xml_diff>
--- a/static/attendance_sheet.xlsx
+++ b/static/attendance_sheet.xlsx
@@ -2797,7 +2797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2811,6 +2811,11 @@
           <t>Name</t>
         </is>
       </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>22-08-2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2821,6 +2826,9 @@
           <t>Abhishek</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2831,6 +2839,9 @@
           <t>Arpan</t>
         </is>
       </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2841,6 +2852,9 @@
           <t>Ashutosh</t>
         </is>
       </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2851,6 +2865,9 @@
           <t>Jatin</t>
         </is>
       </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2861,6 +2878,9 @@
           <t>Jyotiranjan</t>
         </is>
       </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2871,6 +2891,9 @@
           <t>Mohit</t>
         </is>
       </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2881,6 +2904,9 @@
           <t>Pranjal</t>
         </is>
       </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2891,6 +2917,9 @@
           <t>Pranjul</t>
         </is>
       </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2900,6 +2929,9 @@
         <is>
           <t>Tarun</t>
         </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>